<commit_message>
Implemented first version of 3 Previewers
(cherry picked from commit 01f0913ada26fa351d9477106230aa0f630bb2ef)
</commit_message>
<xml_diff>
--- a/DemoData.xlsx
+++ b/DemoData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\WeBuild\ExcelDemo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A32E0499-DBA4-403E-A4D7-8491F1B84FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3A1B2A-AC04-444E-A802-79051F432C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52B9497D-902D-4C21-8B78-8D60B2FBE9FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{52B9497D-902D-4C21-8B78-8D60B2FBE9FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Diagram" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>A</t>
   </si>
@@ -51,6 +52,21 @@
   </si>
   <si>
     <t>D</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Austria</t>
   </si>
 </sst>
 </file>
@@ -86,13 +102,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -103,6 +124,842 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Diagram!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Summary</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Diagram!$A$2:$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Italy</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Germany</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Austria</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Diagram!$B$2:$B$4</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>200000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>50000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-BB4A-4A44-AB16-5C070972621F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>147637</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>33337</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Diagramm 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13DCB199-BF9E-314F-2C74-3E8684789A82}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -117,6 +974,17 @@
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CE229C4A-8C2D-40A6-AAC9-60B6931BBB75}" name="Tabelle2" displayName="Tabelle2" ref="A1:B4" totalsRowShown="0">
+  <autoFilter ref="A1:B4" xr:uid="{CE229C4A-8C2D-40A6-AAC9-60B6931BBB75}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{A7CEE1BD-1110-4C8F-965C-C6CD714AF37C}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{681E5BB9-D929-4D71-B8A5-967DC20F560A}" name="Summary" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -60472,6 +61340,52 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7D80B93-E246-4EF9-8675-D15124AC48AF}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1">
+        <v>50000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{410ca847-c6e0-4f63-8fc9-75ba1ca0f841}" enabled="1" method="Privileged" siteId="{c1345815-7f98-4646-a59b-6629a8bf12ca}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
Added support for pictures
(cherry picked from commit b5a3eaf6542039e6c23e5e9474730c6f79a45d26)
</commit_message>
<xml_diff>
--- a/DemoData.xlsx
+++ b/DemoData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\WeBuild\ExcelDemo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3A1B2A-AC04-444E-A802-79051F432C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAAF7FB2-B01F-48A1-9B14-17060296C5D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{52B9497D-902D-4C21-8B78-8D60B2FBE9FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52B9497D-902D-4C21-8B78-8D60B2FBE9FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>A</t>
   </si>
@@ -68,6 +68,12 @@
   <si>
     <t>Austria</t>
   </si>
+  <si>
+    <t>Joined Cell V</t>
+  </si>
+  <si>
+    <t>Joined cell H</t>
+  </si>
 </sst>
 </file>
 
@@ -82,12 +88,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -102,9 +114,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -203,6 +221,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-963B-43A2-86C9-D5D3E3EBDFC5}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -218,6 +241,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-963B-43A2-86C9-D5D3E3EBDFC5}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -233,6 +261,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-963B-43A2-86C9-D5D3E3EBDFC5}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -923,6 +956,64 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Grafik 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD0220A5-D3D0-225D-9D46-DB06BFC977AB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{837473B0-CC2E-450A-ABE3-18F120FF3D39}">
+              <a1611:picAttrSrcUrl xmlns:a1611="http://schemas.microsoft.com/office/drawing/2016/11/main" r:id="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6972300" y="457200"/>
+          <a:ext cx="6905625" cy="4591050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
@@ -1305,10 +1396,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A91EAC18-5041-4675-AA5B-88504F7BC51F}">
-  <dimension ref="A1:D4001"/>
+  <dimension ref="A1:H4001"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="24" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1322,7 +1416,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1337,7 +1431,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1351,8 +1445,13 @@
         <f>A3+B3+C3</f>
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1367,7 +1466,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1382,7 +1481,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1396,8 +1495,11 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1411,8 +1513,9 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1426,8 +1529,9 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1442,7 +1546,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1457,7 +1561,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1472,7 +1576,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1487,7 +1591,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1502,7 +1606,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1517,7 +1621,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1532,7 +1636,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -61323,6 +61427,10 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="F6:F8"/>
+  </mergeCells>
   <conditionalFormatting sqref="D1:D1048576">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -61334,8 +61442,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>